<commit_message>
Update production static site
</commit_message>
<xml_diff>
--- a/assets/samples/fitness_centers/romania/cards_sample_50.xlsx
+++ b/assets/samples/fitness_centers/romania/cards_sample_50.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="631">
   <si>
     <t>entity_id</t>
   </si>
@@ -202,9 +202,6 @@
     <t>LDI1-RO-FI-9ATT-V0PM-36</t>
   </si>
   <si>
-    <t>LDI1-RO-FI-YQ7A-XVP0-13</t>
-  </si>
-  <si>
     <t>LDI1-RO-FI-G6J3-E1XE-30</t>
   </si>
   <si>
@@ -229,6 +226,9 @@
     <t>LDI1-RO-FI-BD3X-5B3D-50</t>
   </si>
   <si>
+    <t>LDI1-RO-FI-7HSR-6RBK-83</t>
+  </si>
+  <si>
     <t>Fitness 4 All Hunedoara</t>
   </si>
   <si>
@@ -352,9 +352,6 @@
     <t>MY GYM</t>
   </si>
   <si>
-    <t>Extreme</t>
-  </si>
-  <si>
     <t>Sweat - The Light</t>
   </si>
   <si>
@@ -379,12 +376,12 @@
     <t>SHAPE UP STUDIO UNIRII</t>
   </si>
   <si>
+    <t>FITACTIVE București Vitan</t>
+  </si>
+  <si>
     <t>Sală de fitness</t>
   </si>
   <si>
-    <t>Complex sportiv</t>
-  </si>
-  <si>
     <t>Bulevardul Dacia, Hunedoara</t>
   </si>
   <si>
@@ -508,9 +505,6 @@
     <t>Șos. București-Domnești 16</t>
   </si>
   <si>
-    <t>Strada Soldat Ghiță Șerban 15, București</t>
-  </si>
-  <si>
     <t>Bulevardul Iuliu Maniu 6Q, București</t>
   </si>
   <si>
@@ -535,6 +529,9 @@
     <t>Bloc C1, Strada Mămulari 2, blC1, sc 2, parter, București</t>
   </si>
   <si>
+    <t>Calea Vitan 289, București</t>
+  </si>
+  <si>
     <t>331013</t>
   </si>
   <si>
@@ -652,9 +649,6 @@
     <t>077090</t>
   </si>
   <si>
-    <t>515100</t>
-  </si>
-  <si>
     <t>061344</t>
   </si>
   <si>
@@ -673,6 +667,9 @@
     <t>417498</t>
   </si>
   <si>
+    <t>077160</t>
+  </si>
+  <si>
     <t>Hunedoara</t>
   </si>
   <si>
@@ -853,9 +850,6 @@
     <t>44.4031801</t>
   </si>
   <si>
-    <t>44.415376</t>
-  </si>
-  <si>
     <t>44.4347598</t>
   </si>
   <si>
@@ -877,6 +871,9 @@
     <t>44.428577</t>
   </si>
   <si>
+    <t>44.4057611</t>
+  </si>
+  <si>
     <t>22.9081019</t>
   </si>
   <si>
@@ -1000,9 +997,6 @@
     <t>25.9540021</t>
   </si>
   <si>
-    <t>26.1692759</t>
-  </si>
-  <si>
     <t>26.0506442</t>
   </si>
   <si>
@@ -1024,6 +1018,9 @@
     <t>26.1076559</t>
   </si>
   <si>
+    <t>26.1424972</t>
+  </si>
+  <si>
     <t>https://www.fitnesshunedoara.ro/</t>
   </si>
   <si>
@@ -1108,9 +1105,6 @@
     <t>https://www.gymone.ro/</t>
   </si>
   <si>
-    <t>https://csextreme.ro/</t>
-  </si>
-  <si>
     <t>https://sweat.ro/the-light/</t>
   </si>
   <si>
@@ -1129,6 +1123,9 @@
     <t>https://www.shape-up.ro/</t>
   </si>
   <si>
+    <t>https://shop.fitactive.ro/</t>
+  </si>
+  <si>
     <t>+40770316651</t>
   </si>
   <si>
@@ -1243,9 +1240,6 @@
     <t>+40740862273</t>
   </si>
   <si>
-    <t>+40727898822</t>
-  </si>
-  <si>
     <t>+40770642390</t>
   </si>
   <si>
@@ -1267,6 +1261,9 @@
     <t>+40731122100</t>
   </si>
   <si>
+    <t>+40758987111</t>
+  </si>
+  <si>
     <t>office@fitnesshunedoara.ro</t>
   </si>
   <si>
@@ -1321,9 +1318,6 @@
     <t>contact@gymone.ro</t>
   </si>
   <si>
-    <t>office@csextreme.ro</t>
-  </si>
-  <si>
     <t>contact@sweat.ro</t>
   </si>
   <si>
@@ -1336,6 +1330,9 @@
     <t>contact@shape-up.ro</t>
   </si>
   <si>
+    <t>vitan@fitactive.ro</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps/place/Fitness+4+All+Hunedoara/data=!4m7!3m6!1s0x474e8a5883569dd9:0x4005109328c46127!8m2!3d45.7593955!4d22.9081019!16s%2Fg%2F11ggr7gn3y!19sChIJ2Z1Wg1iKTkcRJ2HEKJMQBUA?authuser=0&amp;hl=ro&amp;rclk=1</t>
   </si>
   <si>
@@ -1459,9 +1456,6 @@
     <t>https://www.google.com/maps/place/MY+GYM/@44.4031801,25.9540021,17z/data=!3m1!4b1!4m6!3m5!1s0x40adffa7be8e83cf:0xc10f2b6c97188ae0!8m2!3d44.4031801!4d25.9540021!16s%2Fg%2F11ssfqwz_m?hl=ro&amp;entry=ttu&amp;g_ep=EgoyMDI2MDQxNS4wIKXMDSoASAFQAw%3D%3D</t>
   </si>
   <si>
-    <t>https://www.google.com/maps/place/Extreme/data=!4m7!3m6!1s0x40b1fea17e375841:0x6b39b0673ad64370!8m2!3d44.415376!4d26.1692759!16s%2Fg%2F1td68cgr!19sChIJQVg3fqH-sUARcEPWOmewOWs?authuser=0&amp;hl=ro&amp;rclk=1</t>
-  </si>
-  <si>
     <t>https://www.google.com/maps/place/Sweat+-+The+Light/data=!4m7!3m6!1s0x40b2011c97f84f45:0x5e734955c81e125a!8m2!3d44.4347598!4d26.0506442!16s%2Fg%2F11kfpyfkyl!19sChIJRU_4lxwBskARWhIeyFVJc14?authuser=0&amp;hl=ro&amp;rclk=1</t>
   </si>
   <si>
@@ -1486,6 +1480,9 @@
     <t>https://www.google.com/maps/place/SHAPE+UP+STUDIO+UNIRII/data=!4m7!3m6!1s0x40b1ff3d82c46ec9:0x51ee99160b6c361c!8m2!3d44.428577!4d26.1076559!16s%2Fg%2F11bymsnmd9!19sChIJyW7Egj3_sUARHDZsCxaZ7lE?authuser=0&amp;hl=ro&amp;rclk=1</t>
   </si>
   <si>
+    <t>https://www.google.com/maps/place/FITACTIVE+Bucure%C8%99ti+Vitan/data=!4m7!3m6!1s0x40b1ff9eef1436f7:0xd22a1933c5407872!8m2!3d44.4057611!4d26.1424972!16s%2Fg%2F11vy14t96m!19sChIJ9zYU757_sUARcnhAxTMZKtI?authuser=0&amp;hl=ro&amp;rclk=1</t>
+  </si>
+  <si>
     <t>luni: 08-22; marți: 08-22; miercuri: 08-22; joi: 08-22; vineri: 08-22; sâmbătă: 09-22; duminică: 10-20</t>
   </si>
   <si>
@@ -1585,9 +1582,6 @@
     <t>luni: 06-23; marți: 06-23; miercuri: 06-23; joi: 06-23; vineri: 06-23; sâmbătă: 09-21; duminică: 09-21</t>
   </si>
   <si>
-    <t>luni: 09-00; marți: 09-00; miercuri: 09-00; joi: 09-00; vineri: 09-00; sâmbătă: 09-18; duminică: 09-18</t>
-  </si>
-  <si>
     <t>luni: 06-22; marți: 06-22; miercuri: 06-22; joi: 06-22; vineri: 06-22; sâmbătă: 09-19; duminică: 09-19</t>
   </si>
   <si>
@@ -1744,9 +1738,6 @@
     <t>95</t>
   </si>
   <si>
-    <t>615</t>
-  </si>
-  <si>
     <t>320</t>
   </si>
   <si>
@@ -1762,6 +1753,9 @@
     <t>133</t>
   </si>
   <si>
+    <t>124</t>
+  </si>
+  <si>
     <t>https://www.facebook.com/fitnesshunedoara</t>
   </si>
   <si>
@@ -1858,6 +1852,9 @@
     <t>https://www.instagram.com/shapeupstudio</t>
   </si>
   <si>
+    <t>https://www.instagram.com/fitactivebucuresti_vitan</t>
+  </si>
+  <si>
     <t>https://wa.me/40738711661</t>
   </si>
   <si>
@@ -1907,6 +1904,9 @@
   </si>
   <si>
     <t>https://www.tiktok.com/@18gymromania</t>
+  </si>
+  <si>
+    <t>https://www.tiktok.com/@fitactivebucurestivitan</t>
   </si>
 </sst>
 </file>
@@ -2356,49 +2356,49 @@
         <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="K2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="L2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="N2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="O2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -2412,40 +2412,40 @@
         <v>121</v>
       </c>
       <c r="D3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="N3" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="O3" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="P3" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -2459,40 +2459,40 @@
         <v>121</v>
       </c>
       <c r="D4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="K4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="N4" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="O4" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="P4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -2506,43 +2506,43 @@
         <v>121</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="K5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="L5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="N5" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="O5" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P5" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="6" spans="1:21">
@@ -2556,40 +2556,40 @@
         <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="K6" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="L6" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="N6" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="O6" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="P6" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
     </row>
     <row r="7" spans="1:21">
@@ -2603,52 +2603,52 @@
         <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="K7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="L7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N7" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="O7" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P7" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="8" spans="1:21">
@@ -2662,43 +2662,43 @@
         <v>121</v>
       </c>
       <c r="D8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="L8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="N8" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="O8" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="P8" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="9" spans="1:21">
@@ -2712,52 +2712,52 @@
         <v>121</v>
       </c>
       <c r="D9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="K9" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="N9" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="O9" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="P9" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="10" spans="1:21">
@@ -2771,43 +2771,43 @@
         <v>121</v>
       </c>
       <c r="D10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I10" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K10" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="L10" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="N10" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="O10" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P10" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="11" spans="1:21">
@@ -2821,52 +2821,52 @@
         <v>121</v>
       </c>
       <c r="D11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F11" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G11" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I11" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="K11" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="L11" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="N11" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="O11" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="P11" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="12" spans="1:21">
@@ -2880,34 +2880,34 @@
         <v>121</v>
       </c>
       <c r="D12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="O12" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="P12" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="13" spans="1:21">
@@ -2921,46 +2921,46 @@
         <v>121</v>
       </c>
       <c r="D13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F13" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I13" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="K13" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="L13" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="N13" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="O13" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P13" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="R13" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
     </row>
     <row r="14" spans="1:21">
@@ -2974,49 +2974,49 @@
         <v>121</v>
       </c>
       <c r="D14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="L14" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="N14" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="O14" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P14" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="R14" s="2" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="15" spans="1:21">
@@ -3030,37 +3030,37 @@
         <v>121</v>
       </c>
       <c r="D15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G15" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H15" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I15" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K15" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="N15" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="O15" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="P15" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="16" spans="1:21">
@@ -3074,49 +3074,49 @@
         <v>121</v>
       </c>
       <c r="D16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F16" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G16" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H16" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="K16" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L16" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="N16" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="O16" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P16" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="R16" s="2" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
     </row>
     <row r="17" spans="1:21">
@@ -3130,34 +3130,34 @@
         <v>121</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H17" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I17" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="N17" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="O17" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P17" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="18" spans="1:21">
@@ -3171,40 +3171,40 @@
         <v>121</v>
       </c>
       <c r="D18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G18" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H18" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="I18" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="K18" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="N18" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="O18" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="P18" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="19" spans="1:21">
@@ -3218,52 +3218,52 @@
         <v>121</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E19" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H19" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I19" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="K19" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="N19" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="O19" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="P19" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="U19" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="20" spans="1:21">
@@ -3277,37 +3277,37 @@
         <v>121</v>
       </c>
       <c r="D20" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H20" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I20" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K20" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="N20" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="O20" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="P20" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="21" spans="1:21">
@@ -3321,37 +3321,37 @@
         <v>121</v>
       </c>
       <c r="D21" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E21" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H21" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I21" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="K21" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="N21" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="O21" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P21" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="22" spans="1:21">
@@ -3365,49 +3365,49 @@
         <v>121</v>
       </c>
       <c r="D22" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E22" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H22" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I22" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K22" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="L22" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="N22" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="O22" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P22" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="Q22" s="2" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="R22" s="2" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="23" spans="1:21">
@@ -3421,40 +3421,40 @@
         <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H23" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I23" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="K23" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="N23" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="O23" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P23" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="24" spans="1:21">
@@ -3468,40 +3468,40 @@
         <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E24" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I24" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="K24" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="N24" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="O24" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="P24" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="25" spans="1:21">
@@ -3515,49 +3515,49 @@
         <v>121</v>
       </c>
       <c r="D25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H25" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I25" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="K25" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="N25" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="O25" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="P25" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="R25" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="S25" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="26" spans="1:21">
@@ -3571,34 +3571,34 @@
         <v>121</v>
       </c>
       <c r="D26" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F26" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G26" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H26" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I26" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K26" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="O26" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="P26" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="27" spans="1:21">
@@ -3612,46 +3612,46 @@
         <v>121</v>
       </c>
       <c r="D27" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E27" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F27" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G27" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H27" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I27" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="K27" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L27" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="N27" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="O27" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P27" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="S27" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="28" spans="1:21">
@@ -3665,46 +3665,46 @@
         <v>121</v>
       </c>
       <c r="D28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E28" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F28" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G28" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H28" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I28" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="N28" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="O28" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="P28" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="R28" s="2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="T28" s="2" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="29" spans="1:21">
@@ -3718,46 +3718,46 @@
         <v>121</v>
       </c>
       <c r="D29" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H29" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I29" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="K29" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="N29" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="O29" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="P29" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="Q29" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="S29" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="30" spans="1:21">
@@ -3771,37 +3771,37 @@
         <v>121</v>
       </c>
       <c r="D30" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F30" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G30" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H30" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I30" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="K30" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="N30" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="O30" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="P30" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -3815,43 +3815,43 @@
         <v>121</v>
       </c>
       <c r="D31" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E31" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F31" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G31" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H31" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I31" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="K31" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="L31" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="N31" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="O31" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="P31" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="32" spans="1:21">
@@ -3865,40 +3865,40 @@
         <v>121</v>
       </c>
       <c r="D32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E32" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F32" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G32" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I32" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="K32" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="N32" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="O32" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P32" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="33" spans="1:21">
@@ -3912,49 +3912,49 @@
         <v>121</v>
       </c>
       <c r="D33" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E33" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F33" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G33" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H33" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I33" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="K33" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="L33" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="N33" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="O33" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="P33" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="Q33" s="2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="T33" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="34" spans="1:21">
@@ -3968,43 +3968,43 @@
         <v>121</v>
       </c>
       <c r="D34" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E34" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F34" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G34" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H34" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I34" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="K34" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="L34" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="N34" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="O34" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P34" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="35" spans="1:21">
@@ -4018,46 +4018,46 @@
         <v>121</v>
       </c>
       <c r="D35" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F35" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G35" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H35" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I35" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="K35" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="L35" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="N35" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="O35" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P35" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="Q35" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="T35" s="2" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="36" spans="1:21">
@@ -4071,43 +4071,43 @@
         <v>121</v>
       </c>
       <c r="D36" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E36" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H36" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I36" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="K36" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="N36" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="O36" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P36" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="U36" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="37" spans="1:21">
@@ -4121,49 +4121,49 @@
         <v>121</v>
       </c>
       <c r="D37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E37" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F37" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G37" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H37" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I37" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="K37" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="L37" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="N37" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="O37" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="P37" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="Q37" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="R37" s="2" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
     </row>
     <row r="38" spans="1:21">
@@ -4177,43 +4177,43 @@
         <v>121</v>
       </c>
       <c r="D38" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E38" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F38" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G38" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H38" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I38" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="K38" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="L38" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="N38" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="O38" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="P38" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="39" spans="1:21">
@@ -4227,40 +4227,40 @@
         <v>121</v>
       </c>
       <c r="D39" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E39" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F39" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G39" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H39" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I39" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K39" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="N39" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="O39" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P39" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="Q39" s="2" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="40" spans="1:21">
@@ -4274,34 +4274,34 @@
         <v>121</v>
       </c>
       <c r="D40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E40" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F40" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G40" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I40" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="K40" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="O40" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P40" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="41" spans="1:21">
@@ -4315,34 +4315,34 @@
         <v>121</v>
       </c>
       <c r="D41" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E41" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F41" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G41" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H41" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I41" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="N41" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="O41" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="P41" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="42" spans="1:21">
@@ -4356,37 +4356,37 @@
         <v>121</v>
       </c>
       <c r="D42" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E42" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F42" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G42" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H42" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I42" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K42" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="N42" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="O42" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="P42" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="43" spans="1:21">
@@ -4397,46 +4397,55 @@
         <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D43" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E43" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F43" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G43" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H43" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I43" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="K43" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="L43" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="N43" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="O43" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="P43" t="s">
-        <v>576</v>
+        <v>574</v>
+      </c>
+      <c r="Q43" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="R43" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="T43" s="2" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="44" spans="1:21">
@@ -4450,52 +4459,52 @@
         <v>121</v>
       </c>
       <c r="D44" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E44" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F44" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G44" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H44" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I44" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K44" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="L44" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="N44" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="O44" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="P44" t="s">
-        <v>577</v>
+        <v>541</v>
       </c>
       <c r="Q44" s="2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="R44" s="2" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="T44" s="2" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="45" spans="1:21">
@@ -4509,52 +4518,46 @@
         <v>121</v>
       </c>
       <c r="D45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E45" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F45" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="G45" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H45" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I45" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="K45" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="L45" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="N45" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O45" t="s">
         <v>532</v>
       </c>
       <c r="P45" t="s">
-        <v>543</v>
+        <v>575</v>
       </c>
       <c r="Q45" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="R45" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="T45" s="2" t="s">
-        <v>623</v>
+        <v>594</v>
       </c>
     </row>
     <row r="46" spans="1:21">
@@ -4568,46 +4571,52 @@
         <v>121</v>
       </c>
       <c r="D46" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E46" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F46" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G46" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H46" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I46" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="K46" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="L46" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="N46" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="O46" t="s">
-        <v>534</v>
+        <v>528</v>
       </c>
       <c r="P46" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="Q46" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
+      </c>
+      <c r="R46" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="U46" s="2" t="s">
+        <v>628</v>
       </c>
     </row>
     <row r="47" spans="1:21">
@@ -4621,49 +4630,46 @@
         <v>121</v>
       </c>
       <c r="D47" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E47" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F47" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G47" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H47" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I47" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="K47" t="s">
-        <v>413</v>
-      </c>
-      <c r="L47" t="s">
-        <v>438</v>
+        <v>412</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="N47" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="O47" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="P47" t="s">
-        <v>579</v>
-      </c>
-      <c r="Q47" s="2" t="s">
-        <v>597</v>
+        <v>577</v>
       </c>
       <c r="R47" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
+      </c>
+      <c r="T47" s="2" t="s">
+        <v>623</v>
       </c>
       <c r="U47" s="2" t="s">
         <v>629</v>
@@ -4680,52 +4686,37 @@
         <v>121</v>
       </c>
       <c r="D48" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E48" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F48" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="G48" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="H48" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I48" t="s">
-        <v>332</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="K48" t="s">
-        <v>414</v>
+        <v>331</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="N48" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="O48" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="P48" t="s">
-        <v>580</v>
-      </c>
-      <c r="R48" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="T48" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="U48" s="2" t="s">
-        <v>630</v>
+        <v>578</v>
       </c>
     </row>
-    <row r="49" spans="1:20">
+    <row r="49" spans="1:21">
       <c r="A49" t="s">
         <v>68</v>
       </c>
@@ -4736,37 +4727,40 @@
         <v>121</v>
       </c>
       <c r="D49" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F49" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="G49" t="s">
         <v>230</v>
       </c>
       <c r="H49" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I49" t="s">
-        <v>333</v>
+        <v>332</v>
+      </c>
+      <c r="K49" t="s">
+        <v>413</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="N49" t="s">
-        <v>527</v>
+        <v>491</v>
       </c>
       <c r="O49" t="s">
-        <v>537</v>
+        <v>528</v>
       </c>
       <c r="P49" t="s">
-        <v>581</v>
+        <v>538</v>
       </c>
     </row>
-    <row r="50" spans="1:20">
+    <row r="50" spans="1:21">
       <c r="A50" t="s">
         <v>69</v>
       </c>
@@ -4777,40 +4771,55 @@
         <v>121</v>
       </c>
       <c r="D50" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E50" t="s">
-        <v>218</v>
+        <v>194</v>
       </c>
       <c r="F50" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="G50" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="H50" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I50" t="s">
-        <v>334</v>
+        <v>333</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>368</v>
       </c>
       <c r="K50" t="s">
-        <v>415</v>
+        <v>414</v>
+      </c>
+      <c r="L50" t="s">
+        <v>437</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N50" t="s">
-        <v>492</v>
+        <v>526</v>
       </c>
       <c r="O50" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="P50" t="s">
-        <v>540</v>
+        <v>551</v>
+      </c>
+      <c r="Q50" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="R50" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="T50" s="2" t="s">
+        <v>624</v>
       </c>
     </row>
-    <row r="51" spans="1:20">
+    <row r="51" spans="1:21">
       <c r="A51" t="s">
         <v>70</v>
       </c>
@@ -4821,52 +4830,49 @@
         <v>121</v>
       </c>
       <c r="D51" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E51" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="F51" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G51" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H51" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I51" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K51" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L51" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="N51" t="s">
-        <v>528</v>
+        <v>491</v>
       </c>
       <c r="O51" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="P51" t="s">
-        <v>553</v>
-      </c>
-      <c r="Q51" s="2" t="s">
-        <v>598</v>
+        <v>579</v>
       </c>
       <c r="R51" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="T51" s="2" t="s">
-        <v>625</v>
+        <v>612</v>
+      </c>
+      <c r="U51" s="2" t="s">
+        <v>630</v>
       </c>
     </row>
   </sheetData>
@@ -4984,36 +4990,38 @@
     <hyperlink ref="M42" r:id="rId111"/>
     <hyperlink ref="J43" r:id="rId112"/>
     <hyperlink ref="M43" r:id="rId113"/>
-    <hyperlink ref="J44" r:id="rId114"/>
-    <hyperlink ref="M44" r:id="rId115"/>
-    <hyperlink ref="Q44" r:id="rId116"/>
-    <hyperlink ref="R44" r:id="rId117"/>
-    <hyperlink ref="T44" r:id="rId118"/>
-    <hyperlink ref="J45" r:id="rId119"/>
-    <hyperlink ref="M45" r:id="rId120"/>
-    <hyperlink ref="Q45" r:id="rId121"/>
-    <hyperlink ref="R45" r:id="rId122"/>
-    <hyperlink ref="T45" r:id="rId123"/>
-    <hyperlink ref="J46" r:id="rId124"/>
-    <hyperlink ref="M46" r:id="rId125"/>
-    <hyperlink ref="Q46" r:id="rId126"/>
-    <hyperlink ref="J47" r:id="rId127"/>
-    <hyperlink ref="M47" r:id="rId128"/>
-    <hyperlink ref="Q47" r:id="rId129"/>
-    <hyperlink ref="R47" r:id="rId130"/>
-    <hyperlink ref="U47" r:id="rId131"/>
-    <hyperlink ref="J48" r:id="rId132"/>
-    <hyperlink ref="M48" r:id="rId133"/>
-    <hyperlink ref="R48" r:id="rId134"/>
-    <hyperlink ref="T48" r:id="rId135"/>
-    <hyperlink ref="U48" r:id="rId136"/>
-    <hyperlink ref="M49" r:id="rId137"/>
+    <hyperlink ref="Q43" r:id="rId114"/>
+    <hyperlink ref="R43" r:id="rId115"/>
+    <hyperlink ref="T43" r:id="rId116"/>
+    <hyperlink ref="J44" r:id="rId117"/>
+    <hyperlink ref="M44" r:id="rId118"/>
+    <hyperlink ref="Q44" r:id="rId119"/>
+    <hyperlink ref="R44" r:id="rId120"/>
+    <hyperlink ref="T44" r:id="rId121"/>
+    <hyperlink ref="J45" r:id="rId122"/>
+    <hyperlink ref="M45" r:id="rId123"/>
+    <hyperlink ref="Q45" r:id="rId124"/>
+    <hyperlink ref="J46" r:id="rId125"/>
+    <hyperlink ref="M46" r:id="rId126"/>
+    <hyperlink ref="Q46" r:id="rId127"/>
+    <hyperlink ref="R46" r:id="rId128"/>
+    <hyperlink ref="U46" r:id="rId129"/>
+    <hyperlink ref="J47" r:id="rId130"/>
+    <hyperlink ref="M47" r:id="rId131"/>
+    <hyperlink ref="R47" r:id="rId132"/>
+    <hyperlink ref="T47" r:id="rId133"/>
+    <hyperlink ref="U47" r:id="rId134"/>
+    <hyperlink ref="M48" r:id="rId135"/>
+    <hyperlink ref="M49" r:id="rId136"/>
+    <hyperlink ref="J50" r:id="rId137"/>
     <hyperlink ref="M50" r:id="rId138"/>
-    <hyperlink ref="J51" r:id="rId139"/>
-    <hyperlink ref="M51" r:id="rId140"/>
-    <hyperlink ref="Q51" r:id="rId141"/>
-    <hyperlink ref="R51" r:id="rId142"/>
-    <hyperlink ref="T51" r:id="rId143"/>
+    <hyperlink ref="Q50" r:id="rId139"/>
+    <hyperlink ref="R50" r:id="rId140"/>
+    <hyperlink ref="T50" r:id="rId141"/>
+    <hyperlink ref="J51" r:id="rId142"/>
+    <hyperlink ref="M51" r:id="rId143"/>
+    <hyperlink ref="R51" r:id="rId144"/>
+    <hyperlink ref="U51" r:id="rId145"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>